<commit_message>
v2.9: fix - EMA
</commit_message>
<xml_diff>
--- a/resources/Z571/Z571_codebaseline.xlsx
+++ b/resources/Z571/Z571_codebaseline.xlsx
@@ -426,59 +426,356 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>baseline_month</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>source_month</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>defect_desc</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>baseline_rate</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>source_total_panels</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>G向单亮线</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>0.00048</v>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>B暗点</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>38184</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>G向单暗线</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>0.00345</v>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>G向单亮线</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="E3" t="n">
+        <v>38184</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>S向亮线</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>0.00752</v>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>G向单暗线</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0.00291</v>
+      </c>
+      <c r="E4" t="n">
+        <v>38184</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>G向带状Mura</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>38184</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>G向群亮线</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.00016</v>
+      </c>
+      <c r="E6" t="n">
+        <v>38184</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>S向ELA Mura</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>38184</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>S向亮线</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0.00581</v>
+      </c>
+      <c r="E8" t="n">
+        <v>38184</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>S向单暗线</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>0.00476</v>
+      <c r="D9" t="n">
+        <v>0.00432</v>
+      </c>
+      <c r="E9" t="n">
+        <v>38184</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>S向带状Mura</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>38184</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>常亮白斑</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>38184</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>常暗黑斑Mura</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>38184</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>彩斑Mura</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>38184</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>暗点</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>38184</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>白画面黑斑Mura</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>38184</v>
       </c>
     </row>
   </sheetData>
@@ -527,7 +824,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-29T22:44:24.388738</t>
+          <t>2026-07-03T12:26:19.058561</t>
         </is>
       </c>
     </row>
@@ -551,7 +848,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>missing_codes</t>
+          <t>multiplier_changed</t>
         </is>
       </c>
     </row>
@@ -575,7 +872,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-03</t>
         </is>
       </c>
     </row>
@@ -587,7 +884,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>14</t>
         </is>
       </c>
     </row>
@@ -599,7 +896,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>G3亮点=0.5;G向ELA Mura=0;G向单亮线=0.5;G向单暗线=0.8;S向ELA Mura=0;S向亮线=0.7;大面积亮点=0;孔区跑道Mura=5;常亮白斑=0;彩斑Mura=0.3;暗点=0.7;白画面黑斑Mura=3;群暗点=0.8</t>
+          <t>G向单亮线=0.5;G向单暗线=0.8;S向亮线=0.7</t>
         </is>
       </c>
     </row>

</xml_diff>